<commit_message>
FIX: lint and minor fixes
</commit_message>
<xml_diff>
--- a/xlsx/tests/conditional_formatting/cf_tests.xlsx
+++ b/xlsx/tests/conditional_formatting/cf_tests.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nhatcher/Documents/Excel/cf/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72AAF0F8-FC25-3A48-BFBF-CF63A786D8C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52B979E3-AB03-B74B-9E72-7ED63550FA52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="33600" windowHeight="18580" activeTab="1" xr2:uid="{C26BDA45-4231-CC45-9473-C5FC91335907}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="33600" windowHeight="18580" activeTab="6" xr2:uid="{C26BDA45-4231-CC45-9473-C5FC91335907}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="TimePeriod" sheetId="4" r:id="rId4"/>
     <sheet name="ColorScales3" sheetId="5" r:id="rId5"/>
     <sheet name="ColorScales2" sheetId="6" r:id="rId6"/>
+    <sheet name="stop-if-true" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -317,7 +318,97 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="16">
+  <dxfs count="25">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color theme="3"/>
@@ -396,6 +487,11 @@
       <font>
         <color rgb="FF9C0006"/>
       </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -451,11 +547,6 @@
       <font>
         <color rgb="FF9C0006"/>
       </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -1213,7 +1304,7 @@
       </c>
       <c r="B27" s="1">
         <f ca="1">TODAY()</f>
-        <v>46152</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
@@ -1222,7 +1313,7 @@
       </c>
       <c r="B28" s="1">
         <f ca="1">B27-1</f>
-        <v>46151</v>
+        <v>46158</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
@@ -1231,7 +1322,7 @@
       </c>
       <c r="B29" s="1">
         <f ca="1">B27-1.2</f>
-        <v>46150.8</v>
+        <v>46157.8</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
@@ -1240,7 +1331,7 @@
       </c>
       <c r="B30" s="1">
         <f ca="1">B27-0.8</f>
-        <v>46151.199999999997</v>
+        <v>46158.2</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
@@ -1248,13 +1339,13 @@
         <v>5</v>
       </c>
       <c r="B31" s="1">
-        <f t="shared" ref="B29:B31" ca="1" si="0">B30+10</f>
-        <v>46161.2</v>
+        <f t="shared" ref="B31" ca="1" si="0">B30+10</f>
+        <v>46168.2</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:A7">
-    <cfRule type="cellIs" dxfId="15" priority="20" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="24" priority="20" operator="greaterThan">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1269,8 +1360,14 @@
       </iconSet>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A27:A31">
+    <cfRule type="cellIs" dxfId="23" priority="2" operator="between">
+      <formula>2</formula>
+      <formula>4</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B2:B7">
-    <cfRule type="cellIs" dxfId="14" priority="19" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="19" operator="equal">
       <formula>$B$8</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1284,18 +1381,44 @@
       </iconSet>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B27:B31">
+    <cfRule type="timePeriod" dxfId="21" priority="1" timePeriod="yesterday">
+      <formula>FLOOR(B27,1)=TODAY()-1</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="C2:C8">
-    <cfRule type="duplicateValues" dxfId="13" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D8">
-    <cfRule type="top10" dxfId="12" priority="17" percent="1" rank="10"/>
+    <cfRule type="top10" dxfId="19" priority="17" percent="1" rank="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2:E8 F8">
-    <cfRule type="top10" dxfId="11" priority="15" rank="3"/>
-    <cfRule type="top10" dxfId="10" priority="16" percent="1" rank="10"/>
+    <cfRule type="top10" dxfId="18" priority="15" rank="3"/>
+    <cfRule type="top10" dxfId="17" priority="16" percent="1" rank="10"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E17:E22">
+    <cfRule type="iconSet" priority="5">
+      <iconSet iconSet="3Symbols">
+        <cfvo type="percent" val="0"/>
+        <cfvo type="formula" val="$E$16"/>
+        <cfvo type="formula" val="$E$15"/>
+      </iconSet>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F8">
-    <cfRule type="aboveAverage" dxfId="9" priority="14"/>
+    <cfRule type="aboveAverage" dxfId="16" priority="14"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G17:G22">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="20"/>
+        <cfvo type="formula" val="$G$13"/>
+        <color rgb="FFFF7128"/>
+        <color rgb="FFFFEB84"/>
+        <color theme="7"/>
+      </colorScale>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H8">
     <cfRule type="dataBar" priority="13">
@@ -1359,38 +1482,6 @@
         <color rgb="FFFCFCFF"/>
         <color rgb="FFF8696B"/>
       </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E17:E22">
-    <cfRule type="iconSet" priority="5">
-      <iconSet iconSet="3Symbols">
-        <cfvo type="percent" val="0"/>
-        <cfvo type="formula" val="$E$16"/>
-        <cfvo type="formula" val="$E$15"/>
-      </iconSet>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G17:G22">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="num" val="20"/>
-        <cfvo type="formula" val="$G$13"/>
-        <color rgb="FFFF7128"/>
-        <color rgb="FFFFEB84"/>
-        <color theme="7"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A27:A31">
-    <cfRule type="cellIs" dxfId="8" priority="2" operator="between">
-      <formula>2</formula>
-      <formula>4</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B27:B31">
-    <cfRule type="timePeriod" dxfId="7" priority="1" timePeriod="yesterday">
-      <formula>FLOOR(B27,1)=TODAY()-1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1825,6 +1916,24 @@
       </iconSet>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B10:B12">
+    <cfRule type="iconSet" priority="18">
+      <iconSet>
+        <cfvo type="percent" val="0"/>
+        <cfvo type="percent" val="33"/>
+        <cfvo type="percent" val="67"/>
+      </iconSet>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B16:B18">
+    <cfRule type="iconSet" priority="11">
+      <iconSet iconSet="3Symbols">
+        <cfvo type="percent" val="0"/>
+        <cfvo type="percent" val="33"/>
+        <cfvo type="percent" val="67"/>
+      </iconSet>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="C3:C5">
     <cfRule type="iconSet" priority="21">
       <iconSet iconSet="4Arrows">
@@ -1835,6 +1944,35 @@
       </iconSet>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="C10:C12">
+    <cfRule type="iconSet" priority="17">
+      <iconSet iconSet="3Signs">
+        <cfvo type="percent" val="0"/>
+        <cfvo type="percent" val="33"/>
+        <cfvo type="percent" val="67"/>
+      </iconSet>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C16:C18">
+    <cfRule type="iconSet" priority="12">
+      <iconSet iconSet="3Symbols2">
+        <cfvo type="percent" val="0"/>
+        <cfvo type="percent" val="33"/>
+        <cfvo type="percent" val="67"/>
+      </iconSet>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C22:C26">
+    <cfRule type="iconSet" priority="7">
+      <iconSet iconSet="5Quarters">
+        <cfvo type="percent" val="0"/>
+        <cfvo type="percent" val="20"/>
+        <cfvo type="percent" val="40"/>
+        <cfvo type="percent" val="60"/>
+        <cfvo type="percent" val="80"/>
+      </iconSet>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="D3:D6">
     <cfRule type="iconSet" priority="20">
       <iconSet iconSet="4Arrows">
@@ -1842,6 +1980,25 @@
         <cfvo type="percent" val="25"/>
         <cfvo type="percent" val="50"/>
         <cfvo type="percent" val="75"/>
+      </iconSet>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D10:D13 D16:D18">
+    <cfRule type="iconSet" priority="16">
+      <iconSet iconSet="4RedToBlack">
+        <cfvo type="percent" val="0"/>
+        <cfvo type="percent" val="25"/>
+        <cfvo type="percent" val="50"/>
+        <cfvo type="percent" val="75"/>
+      </iconSet>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D16:D18">
+    <cfRule type="iconSet" priority="13">
+      <iconSet iconSet="3Flags">
+        <cfvo type="percent" val="0"/>
+        <cfvo type="percent" val="33"/>
+        <cfvo type="percent" val="67"/>
       </iconSet>
     </cfRule>
   </conditionalFormatting>
@@ -1856,34 +2013,6 @@
       </iconSet>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B10:B12">
-    <cfRule type="iconSet" priority="18">
-      <iconSet>
-        <cfvo type="percent" val="0"/>
-        <cfvo type="percent" val="33"/>
-        <cfvo type="percent" val="67"/>
-      </iconSet>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C10:C12">
-    <cfRule type="iconSet" priority="17">
-      <iconSet iconSet="3Signs">
-        <cfvo type="percent" val="0"/>
-        <cfvo type="percent" val="33"/>
-        <cfvo type="percent" val="67"/>
-      </iconSet>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D10:D13 D16:D18">
-    <cfRule type="iconSet" priority="16">
-      <iconSet iconSet="4RedToBlack">
-        <cfvo type="percent" val="0"/>
-        <cfvo type="percent" val="25"/>
-        <cfvo type="percent" val="50"/>
-        <cfvo type="percent" val="75"/>
-      </iconSet>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="E10:E12">
     <cfRule type="iconSet" priority="15">
       <iconSet iconSet="3TrafficLights2">
@@ -1893,6 +2022,16 @@
       </iconSet>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="E22:E25">
+    <cfRule type="iconSet" priority="9">
+      <iconSet iconSet="4Rating">
+        <cfvo type="percent" val="0"/>
+        <cfvo type="percent" val="25"/>
+        <cfvo type="percent" val="50"/>
+        <cfvo type="percent" val="75"/>
+      </iconSet>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="F10:F13">
     <cfRule type="iconSet" priority="14">
       <iconSet iconSet="4TrafficLights">
@@ -1900,33 +2039,6 @@
         <cfvo type="percent" val="25"/>
         <cfvo type="percent" val="50"/>
         <cfvo type="percent" val="75"/>
-      </iconSet>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D16:D18">
-    <cfRule type="iconSet" priority="13">
-      <iconSet iconSet="3Flags">
-        <cfvo type="percent" val="0"/>
-        <cfvo type="percent" val="33"/>
-        <cfvo type="percent" val="67"/>
-      </iconSet>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C16:C18">
-    <cfRule type="iconSet" priority="12">
-      <iconSet iconSet="3Symbols2">
-        <cfvo type="percent" val="0"/>
-        <cfvo type="percent" val="33"/>
-        <cfvo type="percent" val="67"/>
-      </iconSet>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B16:B18">
-    <cfRule type="iconSet" priority="11">
-      <iconSet iconSet="3Symbols">
-        <cfvo type="percent" val="0"/>
-        <cfvo type="percent" val="33"/>
-        <cfvo type="percent" val="67"/>
       </iconSet>
     </cfRule>
   </conditionalFormatting>
@@ -1941,31 +2053,26 @@
       </iconSet>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E22:E25">
-    <cfRule type="iconSet" priority="9">
-      <iconSet iconSet="4Rating">
-        <cfvo type="percent" val="0"/>
-        <cfvo type="percent" val="25"/>
-        <cfvo type="percent" val="50"/>
-        <cfvo type="percent" val="75"/>
-      </iconSet>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C22:C26">
-    <cfRule type="iconSet" priority="7">
-      <iconSet iconSet="5Quarters">
-        <cfvo type="percent" val="0"/>
-        <cfvo type="percent" val="20"/>
-        <cfvo type="percent" val="40"/>
-        <cfvo type="percent" val="60"/>
-        <cfvo type="percent" val="80"/>
-      </iconSet>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="iconSet" priority="6" id="{0E392AD6-AB51-6A4F-94C5-F6F97703A21E}">
+            <x14:iconSet iconSet="3Stars">
+              <x14:cfvo type="percent">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="percent">
+                <xm:f>33</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="percent">
+                <xm:f>67</xm:f>
+              </x14:cfvo>
+            </x14:iconSet>
+          </x14:cfRule>
+          <xm:sqref>B22:B24</xm:sqref>
+        </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="iconSet" priority="8" id="{29553C64-4DE1-FA46-8239-15AB24C87652}">
             <x14:iconSet iconSet="5Boxes">
@@ -1987,22 +2094,6 @@
             </x14:iconSet>
           </x14:cfRule>
           <xm:sqref>D22:D26</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="iconSet" priority="6" id="{0E392AD6-AB51-6A4F-94C5-F6F97703A21E}">
-            <x14:iconSet iconSet="3Stars">
-              <x14:cfvo type="percent">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="percent">
-                <xm:f>33</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="percent">
-                <xm:f>67</xm:f>
-              </x14:cfvo>
-            </x14:iconSet>
-          </x14:cfRule>
-          <xm:sqref>B22:B24</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="iconSet" priority="5" id="{819FB2A1-F3AF-C840-92B2-D4F12601191E}">
@@ -2203,17 +2294,17 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="A1:A7">
-    <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="es">
+    <cfRule type="containsText" dxfId="15" priority="3" operator="containsText" text="es">
       <formula>NOT(ISERROR(SEARCH("es",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E1:E12 F1">
-    <cfRule type="endsWith" dxfId="5" priority="2" operator="endsWith" text="y">
+  <conditionalFormatting sqref="F1 E1:E12">
+    <cfRule type="endsWith" dxfId="14" priority="2" operator="endsWith" text="y">
       <formula>RIGHT(E1,LEN("y"))="y"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1:I9">
-    <cfRule type="uniqueValues" dxfId="4" priority="1"/>
+    <cfRule type="uniqueValues" dxfId="13" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2232,15 +2323,15 @@
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <f ca="1">TODAY()</f>
-        <v>46152</v>
+        <v>46159</v>
       </c>
       <c r="B2" s="1">
-        <f t="shared" ref="B2:H2" ca="1" si="0">TODAY()</f>
-        <v>46152</v>
+        <f t="shared" ref="B2:C2" ca="1" si="0">TODAY()</f>
+        <v>46159</v>
       </c>
       <c r="C2" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>46152</v>
+        <v>46159</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -2253,15 +2344,15 @@
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <f ca="1">A2+10</f>
-        <v>46162</v>
+        <v>46169</v>
       </c>
       <c r="B3" s="1">
-        <f t="shared" ref="B3:H3" ca="1" si="1">B2+10</f>
-        <v>46162</v>
+        <f t="shared" ref="B3:C3" ca="1" si="1">B2+10</f>
+        <v>46169</v>
       </c>
       <c r="C3" s="1">
         <f t="shared" ca="1" si="1"/>
-        <v>46162</v>
+        <v>46169</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -2280,7 +2371,7 @@
       </c>
       <c r="C4" s="1">
         <f ca="1">C2+33</f>
-        <v>46185</v>
+        <v>46192</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -2358,22 +2449,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:A6">
-    <cfRule type="timePeriod" dxfId="3" priority="4" timePeriod="yesterday">
+    <cfRule type="timePeriod" dxfId="12" priority="4" timePeriod="yesterday">
       <formula>FLOOR(A2,1)=TODAY()-1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B6">
-    <cfRule type="timePeriod" dxfId="2" priority="3" timePeriod="thisMonth">
+    <cfRule type="timePeriod" dxfId="11" priority="3" timePeriod="thisMonth">
       <formula>AND(MONTH(B2)=MONTH(TODAY()),YEAR(B2)=YEAR(TODAY()))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C6">
-    <cfRule type="timePeriod" dxfId="1" priority="2" timePeriod="nextMonth">
+    <cfRule type="timePeriod" dxfId="10" priority="2" timePeriod="nextMonth">
       <formula>AND(MONTH(C2)=MONTH(EDATE(TODAY(),0+1)),YEAR(C2)=YEAR(EDATE(TODAY(),0+1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1:F12">
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Fe">
+    <cfRule type="containsText" dxfId="9" priority="1" operator="containsText" text="Fe">
       <formula>NOT(ISERROR(SEARCH("Fe",F1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2609,4 +2700,102 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7897AEE9-8CC6-F543-8B43-F8AED7839A06}">
+  <dimension ref="A1:A8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="24.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="43" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A1:A8">
+    <cfRule type="dataBar" priority="5">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63C384"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{4E03578B-7270-EF4A-8CB9-4C085D619BEF}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+    <cfRule type="top10" dxfId="3" priority="3" stopIfTrue="1" percent="1" rank="10"/>
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFFF7128"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="duplicateValues" dxfId="2" priority="2" stopIfTrue="1"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{4E03578B-7270-EF4A-8CB9-4C085D619BEF}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF63C384"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>A1:A8</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
+</worksheet>
 </file>
</xml_diff>